<commit_message>
feat: actualizar plantilla excel
</commit_message>
<xml_diff>
--- a/pesaje/analytica/Report/ActaEntregaTickets-Export-Base.xlsx
+++ b/pesaje/analytica/Report/ActaEntregaTickets-Export-Base.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\projects\minersoft-projects\minersoft\acopio-project-configuration\pesaje\analytica\Report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{598C1E5E-EDA6-4D46-AEC4-35FC6F1847DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA70404C-5CA8-4E71-B071-7EA82B4F09FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -280,12 +280,6 @@
   </cellStyleXfs>
   <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="22" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="22" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -313,6 +307,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="22" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="22" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="24">
@@ -601,16 +601,17 @@
   <dimension ref="A1:AV11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.5546875" style="3" customWidth="1"/>
-    <col min="2" max="2" width="34.33203125" style="3" customWidth="1"/>
-    <col min="3" max="3" width="47.33203125" style="3" customWidth="1"/>
-    <col min="4" max="4" width="17.33203125" style="3" customWidth="1"/>
-    <col min="5" max="5" width="23.88671875" style="3" customWidth="1"/>
-    <col min="6" max="6" width="28.44140625" style="3" customWidth="1"/>
-    <col min="7" max="7" width="25.77734375" style="3" customWidth="1"/>
-    <col min="8" max="9" width="28.5546875" style="3" customWidth="1"/>
-    <col min="10" max="10" width="24.77734375" style="3" customWidth="1"/>
-    <col min="11" max="23" width="24.6640625" style="3" customWidth="1"/>
+    <col min="1" max="1" width="11.5546875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="49.77734375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="47.33203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="17.33203125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="23.88671875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="28.44140625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="55.109375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="15.21875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="16.88671875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="24.77734375" style="1" customWidth="1"/>
+    <col min="11" max="23" width="24.6640625" style="1" customWidth="1"/>
     <col min="24" max="24" width="31.5546875" customWidth="1"/>
     <col min="25" max="25" width="30.21875" customWidth="1"/>
     <col min="26" max="26" width="28" customWidth="1"/>
@@ -627,361 +628,361 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:48" x14ac:dyDescent="0.3">
-      <c r="A1" s="4"/>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4"/>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
-      <c r="N1" s="4"/>
-      <c r="O1" s="4"/>
-      <c r="P1" s="4"/>
-      <c r="Q1" s="4"/>
-      <c r="R1" s="4"/>
-      <c r="S1" s="4"/>
-      <c r="T1" s="4"/>
-      <c r="U1" s="4"/>
-      <c r="V1" s="4"/>
-      <c r="W1" s="4"/>
-      <c r="X1" s="5"/>
-      <c r="Y1" s="5"/>
-      <c r="Z1" s="5"/>
-      <c r="AA1" s="5"/>
-      <c r="AB1" s="5"/>
-      <c r="AC1" s="5"/>
-      <c r="AD1" s="5"/>
-      <c r="AE1" s="5"/>
-      <c r="AF1" s="5"/>
-      <c r="AG1" s="5"/>
-      <c r="AH1" s="5"/>
-      <c r="AI1" s="5"/>
-      <c r="AJ1" s="5"/>
-      <c r="AK1" s="5"/>
-      <c r="AL1" s="5"/>
-      <c r="AM1" s="5"/>
-      <c r="AN1" s="5"/>
-      <c r="AO1" s="5"/>
-      <c r="AP1" s="5"/>
-      <c r="AQ1" s="5"/>
-      <c r="AR1" s="5"/>
-      <c r="AS1" s="5"/>
-      <c r="AT1" s="5"/>
-      <c r="AU1" s="5"/>
-      <c r="AV1" s="5"/>
+      <c r="A1" s="2"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
+      <c r="M1" s="2"/>
+      <c r="N1" s="2"/>
+      <c r="O1" s="2"/>
+      <c r="P1" s="2"/>
+      <c r="Q1" s="2"/>
+      <c r="R1" s="2"/>
+      <c r="S1" s="2"/>
+      <c r="T1" s="2"/>
+      <c r="U1" s="2"/>
+      <c r="V1" s="2"/>
+      <c r="W1" s="2"/>
+      <c r="X1" s="3"/>
+      <c r="Y1" s="3"/>
+      <c r="Z1" s="3"/>
+      <c r="AA1" s="3"/>
+      <c r="AB1" s="3"/>
+      <c r="AC1" s="3"/>
+      <c r="AD1" s="3"/>
+      <c r="AE1" s="3"/>
+      <c r="AF1" s="3"/>
+      <c r="AG1" s="3"/>
+      <c r="AH1" s="3"/>
+      <c r="AI1" s="3"/>
+      <c r="AJ1" s="3"/>
+      <c r="AK1" s="3"/>
+      <c r="AL1" s="3"/>
+      <c r="AM1" s="3"/>
+      <c r="AN1" s="3"/>
+      <c r="AO1" s="3"/>
+      <c r="AP1" s="3"/>
+      <c r="AQ1" s="3"/>
+      <c r="AR1" s="3"/>
+      <c r="AS1" s="3"/>
+      <c r="AT1" s="3"/>
+      <c r="AU1" s="3"/>
+      <c r="AV1" s="3"/>
     </row>
     <row r="2" spans="1:48" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="6"/>
-      <c r="L2" s="4"/>
-      <c r="M2" s="4"/>
-      <c r="N2" s="4"/>
-      <c r="O2" s="4"/>
-      <c r="P2" s="4"/>
-      <c r="Q2" s="4"/>
-      <c r="R2" s="4"/>
-      <c r="S2" s="4"/>
-      <c r="T2" s="4"/>
-      <c r="U2" s="4"/>
-      <c r="V2" s="4"/>
-      <c r="W2" s="4"/>
-      <c r="X2" s="5"/>
-      <c r="Y2" s="5"/>
-      <c r="Z2" s="5"/>
-      <c r="AA2" s="5"/>
-      <c r="AB2" s="5"/>
-      <c r="AC2" s="5"/>
-      <c r="AD2" s="5"/>
-      <c r="AE2" s="5"/>
-      <c r="AF2" s="5"/>
-      <c r="AG2" s="5"/>
-      <c r="AH2" s="5"/>
-      <c r="AI2" s="5"/>
-      <c r="AJ2" s="5"/>
-      <c r="AK2" s="5"/>
-      <c r="AL2" s="5"/>
-      <c r="AM2" s="5"/>
-      <c r="AN2" s="5"/>
-      <c r="AO2" s="5"/>
-      <c r="AP2" s="5"/>
-      <c r="AQ2" s="5"/>
-      <c r="AR2" s="5"/>
-      <c r="AS2" s="5"/>
-      <c r="AT2" s="5"/>
-      <c r="AU2" s="5"/>
-      <c r="AV2" s="5"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="11"/>
+      <c r="G2" s="11"/>
+      <c r="H2" s="11"/>
+      <c r="I2" s="11"/>
+      <c r="J2" s="11"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
+      <c r="N2" s="2"/>
+      <c r="O2" s="2"/>
+      <c r="P2" s="2"/>
+      <c r="Q2" s="2"/>
+      <c r="R2" s="2"/>
+      <c r="S2" s="2"/>
+      <c r="T2" s="2"/>
+      <c r="U2" s="2"/>
+      <c r="V2" s="2"/>
+      <c r="W2" s="2"/>
+      <c r="X2" s="3"/>
+      <c r="Y2" s="3"/>
+      <c r="Z2" s="3"/>
+      <c r="AA2" s="3"/>
+      <c r="AB2" s="3"/>
+      <c r="AC2" s="3"/>
+      <c r="AD2" s="3"/>
+      <c r="AE2" s="3"/>
+      <c r="AF2" s="3"/>
+      <c r="AG2" s="3"/>
+      <c r="AH2" s="3"/>
+      <c r="AI2" s="3"/>
+      <c r="AJ2" s="3"/>
+      <c r="AK2" s="3"/>
+      <c r="AL2" s="3"/>
+      <c r="AM2" s="3"/>
+      <c r="AN2" s="3"/>
+      <c r="AO2" s="3"/>
+      <c r="AP2" s="3"/>
+      <c r="AQ2" s="3"/>
+      <c r="AR2" s="3"/>
+      <c r="AS2" s="3"/>
+      <c r="AT2" s="3"/>
+      <c r="AU2" s="3"/>
+      <c r="AV2" s="3"/>
     </row>
     <row r="3" spans="1:48" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
-      <c r="K3" s="7"/>
-      <c r="L3" s="4"/>
-      <c r="M3" s="4"/>
-      <c r="N3" s="4"/>
-      <c r="O3" s="4"/>
-      <c r="P3" s="4"/>
-      <c r="Q3" s="4"/>
-      <c r="R3" s="4"/>
-      <c r="S3" s="4"/>
-      <c r="T3" s="4"/>
-      <c r="U3" s="4"/>
-      <c r="V3" s="4"/>
-      <c r="W3" s="4"/>
-      <c r="X3" s="5"/>
-      <c r="Y3" s="5"/>
-      <c r="Z3" s="5"/>
-      <c r="AA3" s="5"/>
-      <c r="AB3" s="5"/>
-      <c r="AC3" s="5"/>
-      <c r="AD3" s="5"/>
-      <c r="AE3" s="5"/>
-      <c r="AF3" s="5"/>
-      <c r="AG3" s="5"/>
-      <c r="AH3" s="5"/>
-      <c r="AI3" s="5"/>
-      <c r="AJ3" s="5"/>
-      <c r="AK3" s="5"/>
-      <c r="AL3" s="5"/>
-      <c r="AM3" s="5"/>
-      <c r="AN3" s="5"/>
-      <c r="AO3" s="5"/>
-      <c r="AP3" s="5"/>
-      <c r="AQ3" s="5"/>
-      <c r="AR3" s="5"/>
-      <c r="AS3" s="5"/>
-      <c r="AT3" s="5"/>
-      <c r="AU3" s="5"/>
-      <c r="AV3" s="5"/>
+      <c r="B3" s="12"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="12"/>
+      <c r="G3" s="12"/>
+      <c r="H3" s="12"/>
+      <c r="I3" s="12"/>
+      <c r="J3" s="12"/>
+      <c r="K3" s="5"/>
+      <c r="L3" s="2"/>
+      <c r="M3" s="2"/>
+      <c r="N3" s="2"/>
+      <c r="O3" s="2"/>
+      <c r="P3" s="2"/>
+      <c r="Q3" s="2"/>
+      <c r="R3" s="2"/>
+      <c r="S3" s="2"/>
+      <c r="T3" s="2"/>
+      <c r="U3" s="2"/>
+      <c r="V3" s="2"/>
+      <c r="W3" s="2"/>
+      <c r="X3" s="3"/>
+      <c r="Y3" s="3"/>
+      <c r="Z3" s="3"/>
+      <c r="AA3" s="3"/>
+      <c r="AB3" s="3"/>
+      <c r="AC3" s="3"/>
+      <c r="AD3" s="3"/>
+      <c r="AE3" s="3"/>
+      <c r="AF3" s="3"/>
+      <c r="AG3" s="3"/>
+      <c r="AH3" s="3"/>
+      <c r="AI3" s="3"/>
+      <c r="AJ3" s="3"/>
+      <c r="AK3" s="3"/>
+      <c r="AL3" s="3"/>
+      <c r="AM3" s="3"/>
+      <c r="AN3" s="3"/>
+      <c r="AO3" s="3"/>
+      <c r="AP3" s="3"/>
+      <c r="AQ3" s="3"/>
+      <c r="AR3" s="3"/>
+      <c r="AS3" s="3"/>
+      <c r="AT3" s="3"/>
+      <c r="AU3" s="3"/>
+      <c r="AV3" s="3"/>
     </row>
     <row r="4" spans="1:48" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="6"/>
-      <c r="B4" s="6"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
-      <c r="H4" s="6"/>
-      <c r="I4" s="6"/>
-      <c r="J4" s="6"/>
-      <c r="K4" s="6"/>
-      <c r="L4" s="4"/>
-      <c r="M4" s="4"/>
-      <c r="N4" s="4"/>
-      <c r="O4" s="4"/>
-      <c r="P4" s="4"/>
-      <c r="Q4" s="4"/>
-      <c r="R4" s="4"/>
-      <c r="S4" s="4"/>
-      <c r="T4" s="4"/>
-      <c r="U4" s="4"/>
-      <c r="V4" s="4"/>
-      <c r="W4" s="4"/>
-      <c r="X4" s="5"/>
-      <c r="Y4" s="5"/>
-      <c r="Z4" s="5"/>
-      <c r="AA4" s="5"/>
-      <c r="AB4" s="5"/>
-      <c r="AC4" s="5"/>
-      <c r="AD4" s="5"/>
-      <c r="AE4" s="5"/>
-      <c r="AF4" s="5"/>
-      <c r="AG4" s="5"/>
-      <c r="AH4" s="5"/>
-      <c r="AI4" s="5"/>
-      <c r="AJ4" s="5"/>
-      <c r="AK4" s="5"/>
-      <c r="AL4" s="5"/>
-      <c r="AM4" s="5"/>
-      <c r="AN4" s="5"/>
-      <c r="AO4" s="5"/>
-      <c r="AP4" s="5"/>
-      <c r="AQ4" s="5"/>
-      <c r="AR4" s="5"/>
-      <c r="AS4" s="5"/>
-      <c r="AT4" s="5"/>
-      <c r="AU4" s="5"/>
-      <c r="AV4" s="5"/>
+      <c r="A4" s="4"/>
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="4"/>
+      <c r="H4" s="4"/>
+      <c r="I4" s="4"/>
+      <c r="J4" s="4"/>
+      <c r="K4" s="4"/>
+      <c r="L4" s="2"/>
+      <c r="M4" s="2"/>
+      <c r="N4" s="2"/>
+      <c r="O4" s="2"/>
+      <c r="P4" s="2"/>
+      <c r="Q4" s="2"/>
+      <c r="R4" s="2"/>
+      <c r="S4" s="2"/>
+      <c r="T4" s="2"/>
+      <c r="U4" s="2"/>
+      <c r="V4" s="2"/>
+      <c r="W4" s="2"/>
+      <c r="X4" s="3"/>
+      <c r="Y4" s="3"/>
+      <c r="Z4" s="3"/>
+      <c r="AA4" s="3"/>
+      <c r="AB4" s="3"/>
+      <c r="AC4" s="3"/>
+      <c r="AD4" s="3"/>
+      <c r="AE4" s="3"/>
+      <c r="AF4" s="3"/>
+      <c r="AG4" s="3"/>
+      <c r="AH4" s="3"/>
+      <c r="AI4" s="3"/>
+      <c r="AJ4" s="3"/>
+      <c r="AK4" s="3"/>
+      <c r="AL4" s="3"/>
+      <c r="AM4" s="3"/>
+      <c r="AN4" s="3"/>
+      <c r="AO4" s="3"/>
+      <c r="AP4" s="3"/>
+      <c r="AQ4" s="3"/>
+      <c r="AR4" s="3"/>
+      <c r="AS4" s="3"/>
+      <c r="AT4" s="3"/>
+      <c r="AU4" s="3"/>
+      <c r="AV4" s="3"/>
     </row>
     <row r="5" spans="1:48" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="8"/>
-      <c r="B5" s="8"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="8"/>
-      <c r="F5" s="8"/>
-      <c r="G5" s="8"/>
-      <c r="H5" s="8"/>
-      <c r="I5" s="8"/>
-      <c r="J5" s="8"/>
-      <c r="K5" s="8"/>
+      <c r="A5" s="6"/>
+      <c r="B5" s="6"/>
+      <c r="C5" s="6"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="6"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="6"/>
+      <c r="J5" s="6"/>
+      <c r="K5" s="6"/>
     </row>
     <row r="6" spans="1:48" ht="18" x14ac:dyDescent="0.3">
-      <c r="A6" s="9"/>
-      <c r="B6" s="10" t="s">
+      <c r="A6" s="7"/>
+      <c r="B6" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="10"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="10" t="s">
+      <c r="C6" s="8"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="7"/>
+      <c r="F6" s="7"/>
+      <c r="G6" s="8" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:48" ht="18" x14ac:dyDescent="0.3">
-      <c r="A7" s="9"/>
-      <c r="B7" s="9"/>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="9"/>
-      <c r="J7" s="9"/>
-      <c r="K7" s="9"/>
+      <c r="A7" s="7"/>
+      <c r="B7" s="7"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="7"/>
+      <c r="F7" s="7"/>
+      <c r="G7" s="7"/>
+      <c r="H7" s="7"/>
+      <c r="I7" s="7"/>
+      <c r="J7" s="7"/>
+      <c r="K7" s="7"/>
     </row>
-    <row r="8" spans="1:48" s="12" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="11" t="s">
+    <row r="8" spans="1:48" s="10" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="D8" s="11" t="s">
+      <c r="D8" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="E8" s="11" t="s">
+      <c r="E8" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="F8" s="11" t="s">
+      <c r="F8" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="G8" s="11" t="s">
+      <c r="G8" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="H8" s="11" t="s">
+      <c r="H8" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="I8" s="11" t="s">
+      <c r="I8" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="J8" s="11" t="s">
+      <c r="J8" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="K8" s="11" t="s">
+      <c r="K8" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="L8" s="11" t="s">
+      <c r="L8" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="M8" s="11" t="s">
+      <c r="M8" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="N8" s="11" t="s">
+      <c r="N8" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="O8" s="11" t="s">
+      <c r="O8" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="P8" s="11" t="s">
+      <c r="P8" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="Q8" s="11" t="s">
+      <c r="Q8" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="R8" s="11" t="s">
+      <c r="R8" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="S8" s="11" t="s">
+      <c r="S8" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="T8" s="11" t="s">
+      <c r="T8" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="U8" s="11" t="s">
+      <c r="U8" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="V8" s="11" t="s">
+      <c r="V8" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="W8" s="11" t="s">
+      <c r="W8" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="X8" s="11" t="s">
+      <c r="X8" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="Y8" s="11" t="s">
+      <c r="Y8" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="Z8" s="11" t="s">
+      <c r="Z8" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="AA8" s="11" t="s">
+      <c r="AA8" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="AB8" s="11" t="s">
+      <c r="AB8" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="AC8" s="11" t="s">
+      <c r="AC8" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="AD8" s="11" t="s">
+      <c r="AD8" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="AE8" s="11" t="s">
+      <c r="AE8" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="AF8" s="11" t="s">
+      <c r="AF8" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="AG8" s="11" t="s">
+      <c r="AG8" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="AH8" s="11" t="s">
+      <c r="AH8" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="AI8" s="11" t="s">
+      <c r="AI8" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="AJ8" s="11" t="s">
+      <c r="AJ8" s="9" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:48" s="3" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="9" spans="1:48" s="1" customFormat="1" x14ac:dyDescent="0.3"/>
     <row r="11" spans="1:48" x14ac:dyDescent="0.3">
-      <c r="F11" s="3" t="s">
+      <c r="F11" s="1" t="s">
         <v>39</v>
       </c>
     </row>

</xml_diff>